<commit_message>
etsy: orcamento TDAH em frances (Budget-TDAH.xlsx + guia), traducao do anuncio; formulas sem TEXT sensivel a idioma
- build_fr.py: todas as abas, status e listas em frances; mesmas contas
  conferidas no LibreOffice (2100 / 1228,38 / 98,89 / 622,73 / 207,58 por dia).
- TEXT(x,'#,##0.00') e TEXT(data,'dd mmm') trocados por FIXED(x,2) e por
  contagem de dias: formatos dentro de TEXT mudam com o idioma do Excel.
- Assinaturas: 'Cancel within X day(s)'; imagens refeitas.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01DYz1Azd3FHBSgFnLhXfMUY
</commit_message>
<xml_diff>
--- a/etsy/debt-payoff/Debt-Payoff-Planner.xlsx
+++ b/etsy/debt-payoff/Debt-Payoff-Planner.xlsx
@@ -1216,7 +1216,7 @@
     <row r="10" ht="30" customHeight="1">
       <c r="A10" s="1" t="n"/>
       <c r="B10" s="11">
-        <f>IFERROR("Pay the minimum on every debt, and "&amp;TEXT(INDEX(Debts!$H$6:$H$15,MATCH(1,IF(Debts!$J$10="Snowball",Debts!$F$6:$F$15,Debts!$G$6:$G$15),0)),"#,##0.00")&amp;" on "&amp;INDEX(Debts!$B$6:$B$15,MATCH(1,IF(Debts!$J$10="Snowball",Debts!$F$6:$F$15,Debts!$G$6:$G$15),0))&amp;". That is your focus debt.","Add your debts on the Debts tab.")</f>
+        <f>IFERROR("Pay the minimum on every debt, and "&amp;FIXED(INDEX(Debts!$H$6:$H$15,MATCH(1,IF(Debts!$J$10="Snowball",Debts!$F$6:$F$15,Debts!$G$6:$G$15),0)),2)&amp;" on "&amp;INDEX(Debts!$B$6:$B$15,MATCH(1,IF(Debts!$J$10="Snowball",Debts!$F$6:$F$15,Debts!$G$6:$G$15),0))&amp;". That is your focus debt.","Add your debts on the Debts tab.")</f>
         <v/>
       </c>
       <c r="G10" s="1" t="n"/>
@@ -1291,7 +1291,7 @@
         <v/>
       </c>
       <c r="F13" s="17">
-        <f>IF(E14-E13&gt;0.5,"saves "&amp;TEXT(E14-E13,"#,##0")&amp;" in interest","same interest")</f>
+        <f>IF(E14-E13&gt;0.5,"saves "&amp;FIXED(E14-E13,0)&amp;" in interest","same interest")</f>
         <v/>
       </c>
       <c r="G13" s="1" t="n"/>

</xml_diff>

<commit_message>
etsy: plano de dividas sem cara de IA (ingles e frances, textos simples, fotos novas)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01DYz1Azd3FHBSgFnLhXfMUY
</commit_message>
<xml_diff>
--- a/etsy/debt-payoff/Debt-Payoff-Planner.xlsx
+++ b/etsy/debt-payoff/Debt-Payoff-Planner.xlsx
@@ -141,7 +141,7 @@
       <sz val="13"/>
     </font>
   </fonts>
-  <fills count="8">
+  <fills count="7">
     <fill>
       <patternFill/>
     </fill>
@@ -150,8 +150,8 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00F6F4EF"/>
-        <bgColor rgb="00F6F4EF"/>
+        <fgColor rgb="00FFFFFF"/>
+        <bgColor rgb="00FFFFFF"/>
       </patternFill>
     </fill>
     <fill>
@@ -164,12 +164,6 @@
       <patternFill patternType="solid">
         <fgColor rgb="00FFF4C2"/>
         <bgColor rgb="00FFF4C2"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00FFFFFF"/>
-        <bgColor rgb="00FFFFFF"/>
       </patternFill>
     </fill>
     <fill>
@@ -195,16 +189,16 @@
     </border>
     <border>
       <left style="thin">
-        <color rgb="00D9D4C7"/>
+        <color rgb="00D5DBDB"/>
       </left>
       <right style="thin">
-        <color rgb="00D9D4C7"/>
+        <color rgb="00D5DBDB"/>
       </right>
       <top style="thin">
-        <color rgb="00D9D4C7"/>
+        <color rgb="00D5DBDB"/>
       </top>
       <bottom style="thin">
-        <color rgb="00D9D4C7"/>
+        <color rgb="00D5DBDB"/>
       </bottom>
     </border>
   </borders>
@@ -216,39 +210,39 @@
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="12" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="12" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="4" fontId="13" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="4" fontId="14" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="1" fontId="14" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="167" fontId="15" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="4" fontId="13" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="4" fontId="14" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="1" fontId="14" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="167" fontId="15" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="16" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="17" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="17" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="1" fontId="4" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="1" fontId="4" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="166" fontId="4" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="166" fontId="4" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="4" fontId="4" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="4" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="4" fontId="4" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="4" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="4" fontId="4" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="4" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="4" fontId="5" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="4" fontId="5" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="6" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="4" fontId="7" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="7" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -259,7 +253,7 @@
     <xf numFmtId="0" fontId="9" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="11" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="11" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -380,7 +374,7 @@
               <a:defRPr/>
             </a:pPr>
             <a:r>
-              <a:t>Watch each debt disappear</a:t>
+              <a:t>What you owe on each debt</a:t>
             </a:r>
           </a:p>
         </rich>
@@ -1066,7 +1060,7 @@
       <c r="A2" s="1" t="n"/>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Your way out of debt</t>
+          <t>Your debt payoff plan</t>
         </is>
       </c>
       <c r="C2" s="1" t="n"/>
@@ -1083,7 +1077,7 @@
       <c r="A3" s="1" t="n"/>
       <c r="B3" s="3" t="inlineStr">
         <is>
-          <t>Change the method or the extra amount on the Debts tab: everything updates.</t>
+          <t>Change the method or the extra amount on the Debts tab and everything updates.</t>
         </is>
       </c>
       <c r="C3" s="1" t="n"/>
@@ -4347,11 +4341,11 @@
         </is>
       </c>
       <c r="H6" s="31">
-        <f>IF(Debts!$B$6="","",Debts!$B$6&amp;" · due")</f>
+        <f>IF(Debts!$B$6="","",Debts!$B$6&amp;" (due)")</f>
         <v/>
       </c>
       <c r="I6" s="31">
-        <f>IF(Debts!$B$6="","",Debts!$B$6&amp;" · rem")</f>
+        <f>IF(Debts!$B$6="","",Debts!$B$6&amp;" (rem)")</f>
         <v/>
       </c>
       <c r="J6" s="32">
@@ -4359,11 +4353,11 @@
         <v/>
       </c>
       <c r="K6" s="31">
-        <f>IF(Debts!$B$7="","",Debts!$B$7&amp;" · due")</f>
+        <f>IF(Debts!$B$7="","",Debts!$B$7&amp;" (due)")</f>
         <v/>
       </c>
       <c r="L6" s="31">
-        <f>IF(Debts!$B$7="","",Debts!$B$7&amp;" · rem")</f>
+        <f>IF(Debts!$B$7="","",Debts!$B$7&amp;" (rem)")</f>
         <v/>
       </c>
       <c r="M6" s="32">
@@ -4371,11 +4365,11 @@
         <v/>
       </c>
       <c r="N6" s="31">
-        <f>IF(Debts!$B$8="","",Debts!$B$8&amp;" · due")</f>
+        <f>IF(Debts!$B$8="","",Debts!$B$8&amp;" (due)")</f>
         <v/>
       </c>
       <c r="O6" s="31">
-        <f>IF(Debts!$B$8="","",Debts!$B$8&amp;" · rem")</f>
+        <f>IF(Debts!$B$8="","",Debts!$B$8&amp;" (rem)")</f>
         <v/>
       </c>
       <c r="P6" s="32">
@@ -4383,11 +4377,11 @@
         <v/>
       </c>
       <c r="Q6" s="31">
-        <f>IF(Debts!$B$9="","",Debts!$B$9&amp;" · due")</f>
+        <f>IF(Debts!$B$9="","",Debts!$B$9&amp;" (due)")</f>
         <v/>
       </c>
       <c r="R6" s="31">
-        <f>IF(Debts!$B$9="","",Debts!$B$9&amp;" · rem")</f>
+        <f>IF(Debts!$B$9="","",Debts!$B$9&amp;" (rem)")</f>
         <v/>
       </c>
       <c r="S6" s="32">
@@ -4395,11 +4389,11 @@
         <v/>
       </c>
       <c r="T6" s="31">
-        <f>IF(Debts!$B$10="","",Debts!$B$10&amp;" · due")</f>
+        <f>IF(Debts!$B$10="","",Debts!$B$10&amp;" (due)")</f>
         <v/>
       </c>
       <c r="U6" s="31">
-        <f>IF(Debts!$B$10="","",Debts!$B$10&amp;" · rem")</f>
+        <f>IF(Debts!$B$10="","",Debts!$B$10&amp;" (rem)")</f>
         <v/>
       </c>
       <c r="V6" s="32">
@@ -4407,11 +4401,11 @@
         <v/>
       </c>
       <c r="W6" s="31">
-        <f>IF(Debts!$B$11="","",Debts!$B$11&amp;" · due")</f>
+        <f>IF(Debts!$B$11="","",Debts!$B$11&amp;" (due)")</f>
         <v/>
       </c>
       <c r="X6" s="31">
-        <f>IF(Debts!$B$11="","",Debts!$B$11&amp;" · rem")</f>
+        <f>IF(Debts!$B$11="","",Debts!$B$11&amp;" (rem)")</f>
         <v/>
       </c>
       <c r="Y6" s="32">
@@ -4419,11 +4413,11 @@
         <v/>
       </c>
       <c r="Z6" s="31">
-        <f>IF(Debts!$B$12="","",Debts!$B$12&amp;" · due")</f>
+        <f>IF(Debts!$B$12="","",Debts!$B$12&amp;" (due)")</f>
         <v/>
       </c>
       <c r="AA6" s="31">
-        <f>IF(Debts!$B$12="","",Debts!$B$12&amp;" · rem")</f>
+        <f>IF(Debts!$B$12="","",Debts!$B$12&amp;" (rem)")</f>
         <v/>
       </c>
       <c r="AB6" s="32">
@@ -4431,11 +4425,11 @@
         <v/>
       </c>
       <c r="AC6" s="31">
-        <f>IF(Debts!$B$13="","",Debts!$B$13&amp;" · due")</f>
+        <f>IF(Debts!$B$13="","",Debts!$B$13&amp;" (due)")</f>
         <v/>
       </c>
       <c r="AD6" s="31">
-        <f>IF(Debts!$B$13="","",Debts!$B$13&amp;" · rem")</f>
+        <f>IF(Debts!$B$13="","",Debts!$B$13&amp;" (rem)")</f>
         <v/>
       </c>
       <c r="AE6" s="32">
@@ -4443,11 +4437,11 @@
         <v/>
       </c>
       <c r="AF6" s="31">
-        <f>IF(Debts!$B$14="","",Debts!$B$14&amp;" · due")</f>
+        <f>IF(Debts!$B$14="","",Debts!$B$14&amp;" (due)")</f>
         <v/>
       </c>
       <c r="AG6" s="31">
-        <f>IF(Debts!$B$14="","",Debts!$B$14&amp;" · rem")</f>
+        <f>IF(Debts!$B$14="","",Debts!$B$14&amp;" (rem)")</f>
         <v/>
       </c>
       <c r="AH6" s="32">
@@ -4455,11 +4449,11 @@
         <v/>
       </c>
       <c r="AI6" s="31">
-        <f>IF(Debts!$B$15="","",Debts!$B$15&amp;" · due")</f>
+        <f>IF(Debts!$B$15="","",Debts!$B$15&amp;" (due)")</f>
         <v/>
       </c>
       <c r="AJ6" s="31">
-        <f>IF(Debts!$B$15="","",Debts!$B$15&amp;" · rem")</f>
+        <f>IF(Debts!$B$15="","",Debts!$B$15&amp;" (rem)")</f>
         <v/>
       </c>
       <c r="AK6" s="32">
@@ -31553,11 +31547,11 @@
         </is>
       </c>
       <c r="H6" s="31">
-        <f>IF(Debts!$B$6="","",Debts!$B$6&amp;" · due")</f>
+        <f>IF(Debts!$B$6="","",Debts!$B$6&amp;" (due)")</f>
         <v/>
       </c>
       <c r="I6" s="31">
-        <f>IF(Debts!$B$6="","",Debts!$B$6&amp;" · rem")</f>
+        <f>IF(Debts!$B$6="","",Debts!$B$6&amp;" (rem)")</f>
         <v/>
       </c>
       <c r="J6" s="32">
@@ -31565,11 +31559,11 @@
         <v/>
       </c>
       <c r="K6" s="31">
-        <f>IF(Debts!$B$7="","",Debts!$B$7&amp;" · due")</f>
+        <f>IF(Debts!$B$7="","",Debts!$B$7&amp;" (due)")</f>
         <v/>
       </c>
       <c r="L6" s="31">
-        <f>IF(Debts!$B$7="","",Debts!$B$7&amp;" · rem")</f>
+        <f>IF(Debts!$B$7="","",Debts!$B$7&amp;" (rem)")</f>
         <v/>
       </c>
       <c r="M6" s="32">
@@ -31577,11 +31571,11 @@
         <v/>
       </c>
       <c r="N6" s="31">
-        <f>IF(Debts!$B$8="","",Debts!$B$8&amp;" · due")</f>
+        <f>IF(Debts!$B$8="","",Debts!$B$8&amp;" (due)")</f>
         <v/>
       </c>
       <c r="O6" s="31">
-        <f>IF(Debts!$B$8="","",Debts!$B$8&amp;" · rem")</f>
+        <f>IF(Debts!$B$8="","",Debts!$B$8&amp;" (rem)")</f>
         <v/>
       </c>
       <c r="P6" s="32">
@@ -31589,11 +31583,11 @@
         <v/>
       </c>
       <c r="Q6" s="31">
-        <f>IF(Debts!$B$9="","",Debts!$B$9&amp;" · due")</f>
+        <f>IF(Debts!$B$9="","",Debts!$B$9&amp;" (due)")</f>
         <v/>
       </c>
       <c r="R6" s="31">
-        <f>IF(Debts!$B$9="","",Debts!$B$9&amp;" · rem")</f>
+        <f>IF(Debts!$B$9="","",Debts!$B$9&amp;" (rem)")</f>
         <v/>
       </c>
       <c r="S6" s="32">
@@ -31601,11 +31595,11 @@
         <v/>
       </c>
       <c r="T6" s="31">
-        <f>IF(Debts!$B$10="","",Debts!$B$10&amp;" · due")</f>
+        <f>IF(Debts!$B$10="","",Debts!$B$10&amp;" (due)")</f>
         <v/>
       </c>
       <c r="U6" s="31">
-        <f>IF(Debts!$B$10="","",Debts!$B$10&amp;" · rem")</f>
+        <f>IF(Debts!$B$10="","",Debts!$B$10&amp;" (rem)")</f>
         <v/>
       </c>
       <c r="V6" s="32">
@@ -31613,11 +31607,11 @@
         <v/>
       </c>
       <c r="W6" s="31">
-        <f>IF(Debts!$B$11="","",Debts!$B$11&amp;" · due")</f>
+        <f>IF(Debts!$B$11="","",Debts!$B$11&amp;" (due)")</f>
         <v/>
       </c>
       <c r="X6" s="31">
-        <f>IF(Debts!$B$11="","",Debts!$B$11&amp;" · rem")</f>
+        <f>IF(Debts!$B$11="","",Debts!$B$11&amp;" (rem)")</f>
         <v/>
       </c>
       <c r="Y6" s="32">
@@ -31625,11 +31619,11 @@
         <v/>
       </c>
       <c r="Z6" s="31">
-        <f>IF(Debts!$B$12="","",Debts!$B$12&amp;" · due")</f>
+        <f>IF(Debts!$B$12="","",Debts!$B$12&amp;" (due)")</f>
         <v/>
       </c>
       <c r="AA6" s="31">
-        <f>IF(Debts!$B$12="","",Debts!$B$12&amp;" · rem")</f>
+        <f>IF(Debts!$B$12="","",Debts!$B$12&amp;" (rem)")</f>
         <v/>
       </c>
       <c r="AB6" s="32">
@@ -31637,11 +31631,11 @@
         <v/>
       </c>
       <c r="AC6" s="31">
-        <f>IF(Debts!$B$13="","",Debts!$B$13&amp;" · due")</f>
+        <f>IF(Debts!$B$13="","",Debts!$B$13&amp;" (due)")</f>
         <v/>
       </c>
       <c r="AD6" s="31">
-        <f>IF(Debts!$B$13="","",Debts!$B$13&amp;" · rem")</f>
+        <f>IF(Debts!$B$13="","",Debts!$B$13&amp;" (rem)")</f>
         <v/>
       </c>
       <c r="AE6" s="32">
@@ -31649,11 +31643,11 @@
         <v/>
       </c>
       <c r="AF6" s="31">
-        <f>IF(Debts!$B$14="","",Debts!$B$14&amp;" · due")</f>
+        <f>IF(Debts!$B$14="","",Debts!$B$14&amp;" (due)")</f>
         <v/>
       </c>
       <c r="AG6" s="31">
-        <f>IF(Debts!$B$14="","",Debts!$B$14&amp;" · rem")</f>
+        <f>IF(Debts!$B$14="","",Debts!$B$14&amp;" (rem)")</f>
         <v/>
       </c>
       <c r="AH6" s="32">
@@ -31661,11 +31655,11 @@
         <v/>
       </c>
       <c r="AI6" s="31">
-        <f>IF(Debts!$B$15="","",Debts!$B$15&amp;" · due")</f>
+        <f>IF(Debts!$B$15="","",Debts!$B$15&amp;" (due)")</f>
         <v/>
       </c>
       <c r="AJ6" s="31">
-        <f>IF(Debts!$B$15="","",Debts!$B$15&amp;" · rem")</f>
+        <f>IF(Debts!$B$15="","",Debts!$B$15&amp;" (rem)")</f>
         <v/>
       </c>
       <c r="AK6" s="32">
@@ -60550,7 +60544,7 @@
       <c r="A2" s="1" t="n"/>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Start here: 3 minutes</t>
+          <t>Start here</t>
         </is>
       </c>
       <c r="C2" s="1" t="n"/>
@@ -60560,7 +60554,7 @@
       <c r="A3" s="1" t="n"/>
       <c r="B3" s="3" t="inlineStr">
         <is>
-          <t>Only type in YELLOW cells.</t>
+          <t>Type only in the yellow cells. Everything else is calculated.</t>
         </is>
       </c>
       <c r="C3" s="1" t="n"/>
@@ -60581,7 +60575,7 @@
       </c>
       <c r="C5" s="36" t="inlineStr">
         <is>
-          <t>Debts tab: one line per debt: balance, yearly interest %, minimum payment.</t>
+          <t>Debts tab: one line per debt, with the balance, yearly interest rate and minimum payment.</t>
         </is>
       </c>
       <c r="D5" s="1" t="n"/>
@@ -60601,7 +60595,7 @@
       </c>
       <c r="C7" s="36" t="inlineStr">
         <is>
-          <t>Debts tab: how much EXTRA you can pay every month (even 20 helps), and the first payment month.</t>
+          <t>Debts tab: the extra amount you can pay each month (even 20 helps) and the month of the first payment.</t>
         </is>
       </c>
       <c r="D7" s="1" t="n"/>
@@ -60621,7 +60615,7 @@
       </c>
       <c r="C9" s="36" t="inlineStr">
         <is>
-          <t>Pick a method: Avalanche (least interest) or Snowball (quick wins). The Dashboard compares both.</t>
+          <t>Pick a method: Avalanche pays the least interest, Snowball clears small debts first. The Dashboard compares both.</t>
         </is>
       </c>
       <c r="D9" s="1" t="n"/>
@@ -60636,12 +60630,12 @@
       <c r="A11" s="1" t="n"/>
       <c r="B11" s="35" t="inlineStr">
         <is>
-          <t>★</t>
+          <t>4</t>
         </is>
       </c>
       <c r="C11" s="36" t="inlineStr">
         <is>
-          <t>Dashboard: your debt-free date, and ONE thing to do this month: which debt gets the extra money.</t>
+          <t>Dashboard: your debt-free date, and which debt gets the extra money this month.</t>
         </is>
       </c>
       <c r="D11" s="1" t="n"/>
@@ -60656,12 +60650,12 @@
       <c r="A13" s="1" t="n"/>
       <c r="B13" s="35" t="inlineStr">
         <is>
-          <t>↻</t>
+          <t>5</t>
         </is>
       </c>
       <c r="C13" s="36" t="inlineStr">
         <is>
-          <t>Every month: update the balances from your statements. The plan re-calculates.</t>
+          <t>Each month, update the balances from your statements. The plan is worked out again.</t>
         </is>
       </c>
       <c r="D13" s="1" t="n"/>
@@ -60689,7 +60683,7 @@
       <c r="B17" s="1" t="n"/>
       <c r="C17" s="3" t="inlineStr">
         <is>
-          <t>Snowball and Avalanche tabs show the month-by-month plan. Green cell = the month a debt is gone.</t>
+          <t>The Snowball and Avalanche tabs show the plan month by month. A green cell marks the month a debt is paid off.</t>
         </is>
       </c>
       <c r="D17" s="1" t="n"/>
@@ -60705,7 +60699,7 @@
       <c r="B19" s="1" t="n"/>
       <c r="C19" s="3" t="inlineStr">
         <is>
-          <t>A planning tool, not financial advice. Works in Google Sheets and Microsoft Excel.</t>
+          <t>This is a planning tool and does not give financial advice. Works in Google Sheets and Microsoft Excel.</t>
         </is>
       </c>
       <c r="D19" s="1" t="n"/>

</xml_diff>